<commit_message>
Fix duplicate handling and keep incomplete rows in outputs.
Mark exact duplicates in task 3 as ''äóáëü'' with empty IDs for manual cleanup, and keep task 5 records even when amount is missing.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/lesson13_all_tasks_clean.xlsx
+++ b/lesson13_all_tasks_clean.xlsx
@@ -932,7 +932,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>first_visit</t>
+          <t>первичный визит</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>first_visit</t>
+          <t>первичный визит</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>repeat_visit</t>
+          <t>повторный визит</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>first_visit</t>
+          <t>первичный визит</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>repeat_visit</t>
+          <t>повторный визит</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>first_visit</t>
+          <t>первичный визит</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>repeat_visit</t>
+          <t>повторный визит</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>first_visit</t>
+          <t>первичный визит</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep row 9 in complex output and refresh generated files.
Allow missing status/amount rows in task 5 validation so valid records remain in the final workbook, then regenerate all output Excel files.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/lesson13_all_tasks_clean.xlsx
+++ b/lesson13_all_tasks_clean.xlsx
@@ -1302,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1649,37 +1649,69 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2025-03-25</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Волков Игорь</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>79998889900</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>XTA888888888</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Детейлинг</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>2025-03-31</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Морозова Елена</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>79999990011</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>XTA999999999</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Кузовной ремонт</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="G11" t="n">
         <v>3500</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>

</xml_diff>